<commit_message>
Update bot to use a product catalog and improve user interactions
Replace the initial bot structure with a comprehensive Telegram bot for a product catalog, including features for browsing, ordering, FAQs, and user communication.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 43fb071d-ab89-4fc5-b65c-47960c88221d
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 5f780ed0-75fd-47ec-875d-f295d8a4e50d
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Товары" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,34 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +60,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,70 +446,459 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Категория</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Дозировка</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Цена</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Остаток</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Виалки</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Retatrutide</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>10 mg</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Виалки</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Semaglutide</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>5 mg</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Виалки</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>BPC-157</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Body Protection Compound, 5mg</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>49.99</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TB-500</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Thymosin Beta-4, 5mg</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>59.99</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CJC-1295</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Growth Hormone Releasing Hormone, 2mg</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>39.99</v>
-      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>5 mg</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Виалки</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>TB-500 (Thymosin Beta-4)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>10 mg</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>3800</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Виалки</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>CJC-1295 DAC</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2 mg</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Виалки</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Ipamorelin</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>5 mg</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>1900</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Виалки</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Hexarelin</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2 mg</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Виалки</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Sermorelin</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>10 mg</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>3100</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Виалки</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>GHRP-2</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>5 mg</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Виалки</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>GHRP-6</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>5 mg</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Спреи</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>PT-141 (Bremelanotide)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>10 mg</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Спреи</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Oxytocin Spray</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>100 IU</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>2900</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Расходники</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Вода для инъекций</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>10 ml</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Расходники</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Инсулиновые шприцы U-100</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>1 ml</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Консультация</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Консультация специалиста</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>60 мин</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Remove "Catalog" and "Full Catalog" sections from the product browsing interface
Removes the "Catalog" category and associated handlers, buttons, and data from the product browsing system.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 43fb071d-ab89-4fc5-b65c-47960c88221d
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 09e43fa1-3c29-4173-82b7-ce0124bba71a
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -478,7 +478,6 @@
       <c r="F2" t="n">
         <v>10</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -505,7 +504,6 @@
       <c r="F3" t="n">
         <v>10</v>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -532,7 +530,6 @@
       <c r="F4" t="n">
         <v>10</v>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -559,7 +556,6 @@
       <c r="F5" t="n">
         <v>10</v>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -586,7 +582,6 @@
       <c r="F6" t="n">
         <v>10</v>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -613,7 +608,6 @@
       <c r="F7" t="n">
         <v>10</v>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -640,7 +634,6 @@
       <c r="F8" t="n">
         <v>10</v>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -667,7 +660,6 @@
       <c r="F9" t="n">
         <v>10</v>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -694,7 +686,6 @@
       <c r="F10" t="n">
         <v>10</v>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -721,7 +712,6 @@
       <c r="F11" t="n">
         <v>10</v>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -748,7 +738,6 @@
       <c r="F12" t="n">
         <v>10</v>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -775,7 +764,6 @@
       <c r="F13" t="n">
         <v>10</v>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -802,7 +790,6 @@
       <c r="F14" t="n">
         <v>10</v>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -829,7 +816,6 @@
       <c r="F15" t="n">
         <v>10</v>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -856,7 +842,6 @@
       <c r="F16" t="n">
         <v>10</v>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -883,7 +868,6 @@
       <c r="F17" t="n">
         <v>10</v>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -910,7 +894,6 @@
       <c r="F18" t="n">
         <v>10</v>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -937,7 +920,6 @@
       <c r="F19" t="n">
         <v>10</v>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -964,7 +946,6 @@
       <c r="F20" t="n">
         <v>10</v>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -991,7 +972,6 @@
       <c r="F21" t="n">
         <v>10</v>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1018,7 +998,6 @@
       <c r="F22" t="n">
         <v>10</v>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1045,7 +1024,6 @@
       <c r="F23" t="n">
         <v>10</v>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1072,7 +1050,6 @@
       <c r="F24" t="n">
         <v>10</v>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1080,7 +1057,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Эстетика</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1099,7 +1076,6 @@
       <c r="F25" t="n">
         <v>10</v>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1107,7 +1083,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Эстетика</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1126,7 +1102,6 @@
       <c r="F26" t="n">
         <v>10</v>
       </c>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1153,7 +1128,6 @@
       <c r="F27" t="n">
         <v>10</v>
       </c>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1180,7 +1154,6 @@
       <c r="F28" t="n">
         <v>10</v>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1207,7 +1180,6 @@
       <c r="F29" t="n">
         <v>10</v>
       </c>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1234,7 +1206,6 @@
       <c r="F30" t="n">
         <v>10</v>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1242,7 +1213,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Регенерация</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1261,7 +1232,6 @@
       <c r="F31" t="n">
         <v>10</v>
       </c>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1269,7 +1239,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Регенерация</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1288,7 +1258,6 @@
       <c r="F32" t="n">
         <v>10</v>
       </c>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1315,7 +1284,6 @@
       <c r="F33" t="n">
         <v>10</v>
       </c>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1342,7 +1310,6 @@
       <c r="F34" t="n">
         <v>10</v>
       </c>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1369,7 +1336,6 @@
       <c r="F35" t="n">
         <v>10</v>
       </c>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1396,7 +1362,6 @@
       <c r="F36" t="n">
         <v>10</v>
       </c>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1423,7 +1388,6 @@
       <c r="F37" t="n">
         <v>10</v>
       </c>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1450,7 +1414,6 @@
       <c r="F38" t="n">
         <v>10</v>
       </c>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1477,7 +1440,6 @@
       <c r="F39" t="n">
         <v>10</v>
       </c>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1485,7 +1447,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Долголетие</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1504,7 +1466,6 @@
       <c r="F40" t="n">
         <v>10</v>
       </c>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1512,7 +1473,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Долголетие</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1531,7 +1492,6 @@
       <c r="F41" t="n">
         <v>10</v>
       </c>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1539,7 +1499,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Долголетие</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1558,7 +1518,6 @@
       <c r="F42" t="n">
         <v>10</v>
       </c>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1585,7 +1544,6 @@
       <c r="F43" t="n">
         <v>10</v>
       </c>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1612,7 +1570,6 @@
       <c r="F44" t="n">
         <v>10</v>
       </c>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1620,7 +1577,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Долголетие</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1639,7 +1596,6 @@
       <c r="F45" t="n">
         <v>10</v>
       </c>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1666,7 +1622,6 @@
       <c r="F46" t="n">
         <v>10</v>
       </c>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1693,7 +1648,6 @@
       <c r="F47" t="n">
         <v>10</v>
       </c>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1720,7 +1674,6 @@
       <c r="F48" t="n">
         <v>10</v>
       </c>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1747,7 +1700,6 @@
       <c r="F49" t="n">
         <v>10</v>
       </c>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1774,7 +1726,6 @@
       <c r="F50" t="n">
         <v>10</v>
       </c>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1782,7 +1733,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Рост мышц</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1801,7 +1752,6 @@
       <c r="F51" t="n">
         <v>10</v>
       </c>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1809,7 +1759,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Рост мышц</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1828,7 +1778,6 @@
       <c r="F52" t="n">
         <v>10</v>
       </c>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1836,7 +1785,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Рост мышц</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1855,7 +1804,6 @@
       <c r="F53" t="n">
         <v>10</v>
       </c>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1863,7 +1811,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Рост мышц</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1882,7 +1830,6 @@
       <c r="F54" t="n">
         <v>10</v>
       </c>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1890,7 +1837,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Рост мышц</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1909,7 +1856,6 @@
       <c r="F55" t="n">
         <v>10</v>
       </c>
-      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1917,7 +1863,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Рост мышц</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1936,7 +1882,6 @@
       <c r="F56" t="n">
         <v>10</v>
       </c>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1944,7 +1889,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Контроль веса</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1963,7 +1908,6 @@
       <c r="F57" t="n">
         <v>10</v>
       </c>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1971,7 +1915,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Контроль веса</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1990,7 +1934,6 @@
       <c r="F58" t="n">
         <v>10</v>
       </c>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1998,7 +1941,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Контроль веса</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2017,7 +1960,6 @@
       <c r="F59" t="n">
         <v>10</v>
       </c>
-      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2044,7 +1986,6 @@
       <c r="F60" t="n">
         <v>10</v>
       </c>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2071,7 +2012,6 @@
       <c r="F61" t="n">
         <v>10</v>
       </c>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2098,7 +2038,6 @@
       <c r="F62" t="n">
         <v>10</v>
       </c>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2125,7 +2064,6 @@
       <c r="F63" t="n">
         <v>10</v>
       </c>
-      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2133,7 +2071,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Долголетие</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2152,7 +2090,6 @@
       <c r="F64" t="n">
         <v>10</v>
       </c>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2160,7 +2097,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Долголетие</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2179,7 +2116,6 @@
       <c r="F65" t="n">
         <v>10</v>
       </c>
-      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2187,7 +2123,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Долголетие</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2206,7 +2142,6 @@
       <c r="F66" t="n">
         <v>10</v>
       </c>
-      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2214,7 +2149,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Контроль веса</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2233,7 +2168,6 @@
       <c r="F67" t="n">
         <v>10</v>
       </c>
-      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2241,7 +2175,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Контроль веса</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2260,7 +2194,6 @@
       <c r="F68" t="n">
         <v>10</v>
       </c>
-      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2287,7 +2220,6 @@
       <c r="F69" t="n">
         <v>10</v>
       </c>
-      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2314,7 +2246,6 @@
       <c r="F70" t="n">
         <v>10</v>
       </c>
-      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2322,7 +2253,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Контроль веса</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2341,7 +2272,6 @@
       <c r="F71" t="n">
         <v>10</v>
       </c>
-      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2349,7 +2279,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Контроль веса</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2368,7 +2298,6 @@
       <c r="F72" t="n">
         <v>10</v>
       </c>
-      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2395,7 +2324,6 @@
       <c r="F73" t="n">
         <v>10</v>
       </c>
-      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2422,7 +2350,6 @@
       <c r="F74" t="n">
         <v>10</v>
       </c>
-      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2449,7 +2376,6 @@
       <c r="F75" t="n">
         <v>10</v>
       </c>
-      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2476,7 +2402,6 @@
       <c r="F76" t="n">
         <v>10</v>
       </c>
-      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2503,7 +2428,6 @@
       <c r="F77" t="n">
         <v>10</v>
       </c>
-      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2530,7 +2454,6 @@
       <c r="F78" t="n">
         <v>10</v>
       </c>
-      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2557,7 +2480,6 @@
       <c r="F79" t="n">
         <v>10</v>
       </c>
-      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2584,7 +2506,6 @@
       <c r="F80" t="n">
         <v>10</v>
       </c>
-      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2611,7 +2532,6 @@
       <c r="F81" t="n">
         <v>10</v>
       </c>
-      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2638,7 +2558,6 @@
       <c r="F82" t="n">
         <v>10</v>
       </c>
-      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2665,7 +2584,6 @@
       <c r="F83" t="n">
         <v>10</v>
       </c>
-      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2673,7 +2591,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Регенерация</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2692,7 +2610,6 @@
       <c r="F84" t="n">
         <v>10</v>
       </c>
-      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2719,7 +2636,6 @@
       <c r="F85" t="n">
         <v>10</v>
       </c>
-      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2746,7 +2662,6 @@
       <c r="F86" t="n">
         <v>10</v>
       </c>
-      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2754,7 +2669,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Регенерация</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2773,7 +2688,6 @@
       <c r="F87" t="n">
         <v>10</v>
       </c>
-      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2781,7 +2695,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Регенерация</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2800,7 +2714,6 @@
       <c r="F88" t="n">
         <v>10</v>
       </c>
-      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -2808,7 +2721,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Когнитивное</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2827,7 +2740,6 @@
       <c r="F89" t="n">
         <v>10</v>
       </c>
-      <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -2835,7 +2747,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Когнитивное</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2854,7 +2766,6 @@
       <c r="F90" t="n">
         <v>10</v>
       </c>
-      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2881,7 +2792,6 @@
       <c r="F91" t="n">
         <v>10</v>
       </c>
-      <c r="G91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -2908,7 +2818,6 @@
       <c r="F92" t="n">
         <v>10</v>
       </c>
-      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -2935,7 +2844,6 @@
       <c r="F93" t="n">
         <v>10</v>
       </c>
-      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -2962,7 +2870,6 @@
       <c r="F94" t="n">
         <v>10</v>
       </c>
-      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -2989,7 +2896,6 @@
       <c r="F95" t="n">
         <v>10</v>
       </c>
-      <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -3016,7 +2922,6 @@
       <c r="F96" t="n">
         <v>10</v>
       </c>
-      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -3024,7 +2929,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Когнитивное</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3043,7 +2948,6 @@
       <c r="F97" t="n">
         <v>10</v>
       </c>
-      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -3070,7 +2974,6 @@
       <c r="F98" t="n">
         <v>10</v>
       </c>
-      <c r="G98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -3097,7 +3000,6 @@
       <c r="F99" t="n">
         <v>10</v>
       </c>
-      <c r="G99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -3124,7 +3026,6 @@
       <c r="F100" t="n">
         <v>10</v>
       </c>
-      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -3151,7 +3052,6 @@
       <c r="F101" t="n">
         <v>10</v>
       </c>
-      <c r="G101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -3178,7 +3078,6 @@
       <c r="F102" t="n">
         <v>10</v>
       </c>
-      <c r="G102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -3186,7 +3085,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Рост мышц</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -3205,7 +3104,6 @@
       <c r="F103" t="n">
         <v>10</v>
       </c>
-      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -3213,7 +3111,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Рост мышц</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3232,7 +3130,6 @@
       <c r="F104" t="n">
         <v>10</v>
       </c>
-      <c r="G104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -3240,7 +3137,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Каталог</t>
+          <t>Эстетика</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3259,7 +3156,6 @@
       <c r="F105" t="n">
         <v>10</v>
       </c>
-      <c r="G105" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>